<commit_message>
chore: clean up sample data and extend workbook
- Remove redundant CSV files (keep only messy_data.csv for testing)
- Extend sample_workbook.xlsx with 8 sheets: Sales, Inventory, Targets,
  Employees, Customers, Expenses, Revenue, Projects
- Update data generation script with comprehensive business datasets
</commit_message>
<xml_diff>
--- a/data/sample_workbook.xlsx
+++ b/data/sample_workbook.xlsx
@@ -6,6 +6,11 @@
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
     <sheet name="Inventory" sheetId="2" r:id="rId2"/>
     <sheet name="Targets" sheetId="3" r:id="rId3"/>
+    <sheet name="Employees" sheetId="4" r:id="rId4"/>
+    <sheet name="Customers" sheetId="5" r:id="rId5"/>
+    <sheet name="Expenses" sheetId="6" r:id="rId6"/>
+    <sheet name="Revenue" sheetId="7" r:id="rId7"/>
+    <sheet name="Projects" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -1063,4 +1068,1430 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Employee ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Department</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Role</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Hire Date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EMP001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Alice Chen</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Senior Developer</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2021-03-15</v>
+      </c>
+      <c r="F2">
+        <v>125000</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Bob Martinez</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Account Executive</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2022-06-01</v>
+      </c>
+      <c r="F3">
+        <v>85000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EMP003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Carol White</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Marketing Manager</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2020-09-20</v>
+      </c>
+      <c r="F4">
+        <v>95000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EMP004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Daniel Kim</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D5" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2023-01-10</v>
+      </c>
+      <c r="F5">
+        <v>110000</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>EMP005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Eva Johnson</v>
+      </c>
+      <c r="C6" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D6" t="str">
+        <v>HR Specialist</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2021-11-05</v>
+      </c>
+      <c r="F6">
+        <v>72000</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>EMP006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Frank Lee</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Finance</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Financial Analyst</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2022-04-18</v>
+      </c>
+      <c r="F7">
+        <v>88000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>EMP007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Grace Park</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Junior Developer</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2024-02-01</v>
+      </c>
+      <c r="F8">
+        <v>75000</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Henry Zhao</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Sales Director</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2019-07-22</v>
+      </c>
+      <c r="F9">
+        <v>140000</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>EMP009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ivy Brown</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Support</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Support Lead</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2020-12-10</v>
+      </c>
+      <c r="F10">
+        <v>68000</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>EMP010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Jack Wilson</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2018-05-30</v>
+      </c>
+      <c r="F11">
+        <v>155000</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Customer ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Company Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Contact</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Industry</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Annual Revenue</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>CUST001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>TechCorp Inc</v>
+      </c>
+      <c r="C2" t="str">
+        <v>John Smith</v>
+      </c>
+      <c r="D2" t="str">
+        <v>john@techcorp.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Technology</v>
+      </c>
+      <c r="G2">
+        <v>5000000</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>CUST002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Global Retail</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Sarah Johnson</v>
+      </c>
+      <c r="D3" t="str">
+        <v>sarah@globalretail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="G3">
+        <v>12000000</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>CUST003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>HealthFirst</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Michael Brown</v>
+      </c>
+      <c r="D4" t="str">
+        <v>michael@healthfirst.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Healthcare</v>
+      </c>
+      <c r="G4">
+        <v>8500000</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>CUST004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>EduLearn</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Emily Davis</v>
+      </c>
+      <c r="D5" t="str">
+        <v>emily@edulearn.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>UK</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Education</v>
+      </c>
+      <c r="G5">
+        <v>2500000</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>CUST005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>FinanceHub</v>
+      </c>
+      <c r="C6" t="str">
+        <v>David Wilson</v>
+      </c>
+      <c r="D6" t="str">
+        <v>david@financehub.com</v>
+      </c>
+      <c r="E6" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Finance</v>
+      </c>
+      <c r="G6">
+        <v>25000000</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>CUST006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>GreenEnergy</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Lisa Taylor</v>
+      </c>
+      <c r="D7" t="str">
+        <v>lisa@greenenergy.com</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Energy</v>
+      </c>
+      <c r="G7">
+        <v>15000000</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>CUST007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>AutoDrive</v>
+      </c>
+      <c r="C8" t="str">
+        <v>James Anderson</v>
+      </c>
+      <c r="D8" t="str">
+        <v>james@autodrive.com</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Automotive</v>
+      </c>
+      <c r="G8">
+        <v>45000000</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>CUST008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>FoodWorks</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Amanda Martinez</v>
+      </c>
+      <c r="D9" t="str">
+        <v>amanda@foodworks.com</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Mexico</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Food &amp; Beverage</v>
+      </c>
+      <c r="G9">
+        <v>6000000</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Inactive</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>CUST009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MediaMax</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Robert Garcia</v>
+      </c>
+      <c r="D10" t="str">
+        <v>robert@mediamax.com</v>
+      </c>
+      <c r="E10" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Media</v>
+      </c>
+      <c r="G10">
+        <v>3500000</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>CUST010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>BuildRight</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Jennifer Lee</v>
+      </c>
+      <c r="D11" t="str">
+        <v>jennifer@buildright.com</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Construction</v>
+      </c>
+      <c r="G11">
+        <v>18000000</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Expense ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Department</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EXP001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2024-01-05</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Client visit - NYC</v>
+      </c>
+      <c r="E2">
+        <v>1250</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EXP002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2024-01-08</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Software</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Annual license renewal</v>
+      </c>
+      <c r="E3">
+        <v>5400</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EXP003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2024-01-12</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Trade show booth</v>
+      </c>
+      <c r="E4">
+        <v>8500</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EXP004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2024-01-15</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Q1 supplies order</v>
+      </c>
+      <c r="E5">
+        <v>890.5</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Operations</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>EXP005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2024-01-18</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Training</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Team certification course</v>
+      </c>
+      <c r="E6">
+        <v>3200</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>EXP006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2024-01-22</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Conference attendance</v>
+      </c>
+      <c r="E7">
+        <v>2100</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>EXP007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2024-01-25</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Equipment</v>
+      </c>
+      <c r="D8" t="str">
+        <v>New monitors x5</v>
+      </c>
+      <c r="E8">
+        <v>1750</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>EXP008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2024-02-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Consulting</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Security audit</v>
+      </c>
+      <c r="E9">
+        <v>12000</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>EXP009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2024-02-05</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Digital ad campaign</v>
+      </c>
+      <c r="E10">
+        <v>15000</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>EXP010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2024-02-10</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Customer onboarding trip</v>
+      </c>
+      <c r="E11">
+        <v>980</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Support</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Product Line</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Channel</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Units Sold</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Revenue</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Cost</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Profit</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D2">
+        <v>145</v>
+      </c>
+      <c r="E2">
+        <v>43500</v>
+      </c>
+      <c r="F2">
+        <v>29000</v>
+      </c>
+      <c r="G2">
+        <v>14500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="D3">
+        <v>32</v>
+      </c>
+      <c r="E3">
+        <v>15800</v>
+      </c>
+      <c r="F3">
+        <v>9500</v>
+      </c>
+      <c r="G3">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="D4">
+        <v>89</v>
+      </c>
+      <c r="E4">
+        <v>26700</v>
+      </c>
+      <c r="F4">
+        <v>17800</v>
+      </c>
+      <c r="G4">
+        <v>8900</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2024-01-08</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D5">
+        <v>178</v>
+      </c>
+      <c r="E5">
+        <v>53400</v>
+      </c>
+      <c r="F5">
+        <v>35600</v>
+      </c>
+      <c r="G5">
+        <v>17800</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2024-01-08</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D6">
+        <v>45</v>
+      </c>
+      <c r="E6">
+        <v>22500</v>
+      </c>
+      <c r="F6">
+        <v>13500</v>
+      </c>
+      <c r="G6">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2024-01-08</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="D7">
+        <v>28</v>
+      </c>
+      <c r="E7">
+        <v>14000</v>
+      </c>
+      <c r="F7">
+        <v>8400</v>
+      </c>
+      <c r="G7">
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2024-01-15</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D8">
+        <v>201</v>
+      </c>
+      <c r="E8">
+        <v>60300</v>
+      </c>
+      <c r="F8">
+        <v>40200</v>
+      </c>
+      <c r="G8">
+        <v>20100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2024-01-15</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="D9">
+        <v>95</v>
+      </c>
+      <c r="E9">
+        <v>28500</v>
+      </c>
+      <c r="F9">
+        <v>19000</v>
+      </c>
+      <c r="G9">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2024-01-15</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D10">
+        <v>52</v>
+      </c>
+      <c r="E10">
+        <v>26000</v>
+      </c>
+      <c r="F10">
+        <v>15600</v>
+      </c>
+      <c r="G10">
+        <v>10400</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2024-01-22</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D11">
+        <v>189</v>
+      </c>
+      <c r="E11">
+        <v>56700</v>
+      </c>
+      <c r="F11">
+        <v>37800</v>
+      </c>
+      <c r="G11">
+        <v>18900</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2024-01-22</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="D12">
+        <v>41</v>
+      </c>
+      <c r="E12">
+        <v>20500</v>
+      </c>
+      <c r="F12">
+        <v>12300</v>
+      </c>
+      <c r="G12">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2024-01-29</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D13">
+        <v>215</v>
+      </c>
+      <c r="E13">
+        <v>64500</v>
+      </c>
+      <c r="F13">
+        <v>43000</v>
+      </c>
+      <c r="G13">
+        <v>21500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2024-01-29</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D14">
+        <v>58</v>
+      </c>
+      <c r="E14">
+        <v>29000</v>
+      </c>
+      <c r="F14">
+        <v>17400</v>
+      </c>
+      <c r="G14">
+        <v>11600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2024-01-29</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Electronics</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Retail</v>
+      </c>
+      <c r="D15">
+        <v>102</v>
+      </c>
+      <c r="E15">
+        <v>30600</v>
+      </c>
+      <c r="F15">
+        <v>20400</v>
+      </c>
+      <c r="G15">
+        <v>10200</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Project ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Project Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Client</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Start Date</v>
+      </c>
+      <c r="E1" t="str">
+        <v>End Date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Budget</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Spent</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PRJ001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Website Redesign</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TechCorp Inc</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2024-01-15</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2024-04-30</v>
+      </c>
+      <c r="F2">
+        <v>75000</v>
+      </c>
+      <c r="G2">
+        <v>45000</v>
+      </c>
+      <c r="H2" t="str">
+        <v>In Progress</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PRJ002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Mobile App v2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Global Retail</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2024-02-01</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2024-07-31</v>
+      </c>
+      <c r="F3">
+        <v>150000</v>
+      </c>
+      <c r="G3">
+        <v>62000</v>
+      </c>
+      <c r="H3" t="str">
+        <v>In Progress</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PRJ003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Data Migration</v>
+      </c>
+      <c r="C4" t="str">
+        <v>HealthFirst</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2023-11-01</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2024-02-28</v>
+      </c>
+      <c r="F4">
+        <v>95000</v>
+      </c>
+      <c r="G4">
+        <v>92000</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PRJ004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CRM Integration</v>
+      </c>
+      <c r="C5" t="str">
+        <v>FinanceHub</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2024-06-30</v>
+      </c>
+      <c r="F5">
+        <v>55000</v>
+      </c>
+      <c r="G5">
+        <v>12000</v>
+      </c>
+      <c r="H5" t="str">
+        <v>In Progress</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PRJ005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Security Upgrade</v>
+      </c>
+      <c r="C6" t="str">
+        <v>EduLearn</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2024-01-10</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2024-03-15</v>
+      </c>
+      <c r="F6">
+        <v>40000</v>
+      </c>
+      <c r="G6">
+        <v>38500</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Completed</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PRJ006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Analytics Dashboard</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MediaMax</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2024-02-15</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2024-05-31</v>
+      </c>
+      <c r="F7">
+        <v>85000</v>
+      </c>
+      <c r="G7">
+        <v>28000</v>
+      </c>
+      <c r="H7" t="str">
+        <v>In Progress</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>PRJ007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>API Development</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AutoDrive</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2024-04-01</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2024-09-30</v>
+      </c>
+      <c r="F8">
+        <v>120000</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Planning</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PRJ008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Cloud Migration</v>
+      </c>
+      <c r="C9" t="str">
+        <v>GreenEnergy</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2023-09-01</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2024-01-31</v>
+      </c>
+      <c r="F9">
+        <v>200000</v>
+      </c>
+      <c r="G9">
+        <v>195000</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Completed</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>